<commit_message>
Update client pages and refine termination planning logic
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/reports/broker-contacts-merged-2026-08-26.xlsx
+++ b/reports/broker-contacts-merged-2026-08-26.xlsx
@@ -485,7 +485,7 @@
         <v/>
       </c>
       <c r="M2" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="N2" t="str">
         <v>2026-09-30</v>
@@ -2601,7 +2601,7 @@
         <v>S-216 Consulting Radiologists</v>
       </c>
       <c r="C17" t="str">
-        <v>has_broker set false, Kellie Haehnel (kellie.haehnel@crlmed.com, corrected from crimed) recorded as the direct client contact, is_active set false and termination date 2026-09-30. Setting is_active false is what marks the status TERMINATED and takes them out of the overdue renewal queue. Note it also removes them from active-client views about five weeks before the termination date.</v>
+        <v>has_broker set false, Kellie Haehnel (kellie.haehnel@crlmed.com, corrected from crimed) recorded as the direct client contact, and termination date 2026-09-30. is_active stays TRUE on purpose: the termination date alone now drives state. S-216 computes as TERMINATING, so the renewal is suppressed immediately while the client stays active and visible, PPRs keep generating and run-out claims keep importing through 2026-12-31.</v>
       </c>
     </row>
     <row r="18">

</xml_diff>